<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.001-07 Nino dit stop et s'éloigne
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.001-07.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.001-07.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le câlin de la cour</t>
+          <t>Nino dit stop et s'éloigne</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cour</t>
+          <t>cour de récréation, marelle, craie, cases, poussière, soleil, caillou</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, Chouchou, papa</t>
+          <t>Nino, Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino joue dans la cour. Chouchou le serre trop fort. Nino dit stop, s'éloigne vers papa sur le banc. Le seau sonne plus loin.</t>
+          <t>Un trait rose s'étire sur le sol chaud. Sur une case, un éclat de marelle luit. Nino veut jouer, maintenant. Aniss serre trop. Sourire parti. Papa s'accroupit. Stop, recule. Merci vécu. Deuxième ruse : le caillou glisse. Il dit stop, recule. Un éclat de marelle tient sur la case.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les pierres de la cour sont froides. Un linge rouge bouge au vent. Un seau en métal sonne. Ça sent le café, près de la porte. Papa ouvre la porte de la cuisine. Tu as entendu le seau, Nino ? Oui, papa. Ça sonne. Le vent le touche. Un banc de bois attend au soleil. En ce moment, Nino joue. Chouchou joue avec lui. Ils sont dans la cour. Chouchou fait un gros câlin. Le câlin est trop fort. Nino est inquiet. C'est trop près. Sa poitrine est coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Nino recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le banc. Papa est l'adulte sur le banc. Papa, c'était trop. Je t'ai entendu. Tu as dit stop. Bravo, Nino. Tu as fait un pas vers le banc. Tu veux ta main dans ma main ? Oui, papa. Nino pose sa main dans la main de papa. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Chouchou pousse le seau tout doucement. Le seau sonne plus loin. La cour redevient calme. Le linge rouge claque une fois. Puis il se calme. Tu as vu le linge ? Oui. Il est rouge. Les pierres se réchauffent. Nino pose un pied dessus. Ce n'est plus froid. On reste sur le banc un moment ? Oui, papa.</t>
+          <t>Un trait rose s'étire sur le sol chaud. Il est long, papa. Tu le vois, le trait ? Oui, papa. La poussière de craie pique le nez. J'ai tracé la marelle. Elle est grande, maman. Maman pose le caillou plat. Le caillou est chaud, un peu lisse. Il est chaud. Tu le touches, Nino ? Oui, du doigt. Sur une case, un éclat de marelle luit. Il brille, maman. Tu le vois, sur la case ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur la craie. La craie gratte un peu. Elle gratte, papa. Tu t'accroupis, Nino ? Un peu. Une miette de craie dort au bord. Une miette, maman. Elle est sèche ? Oui. Le vent soulève un peu de poussière. Ça chatouille, papa. Tu l'entends, le vent ? Oui, il souffle. Une feuille tourne près des cases. Elle tourne. C'est le vent. Les pieds de Nino tapent le sol. Mes pieds, papa. Tu es bien prêt, Nino ? Oui, papa. Le sol de la marelle est rêche. Il est rêche. Aniss arrive près des cases. Ses baskets tapent la poussière. La marelle. Tu viens, Aniss ? Oui. Maman tend le caillou. Il tient chaud dans la paume. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. En ce moment, Nino lève le caillou. Tu le lances, Nino ? Oui, maman. Le caillou tape la première case. Moi aussi ! Aniss ouvre les bras tout grand. Il serre Nino très fort. Oh. Le sourire de Nino disparaît. Dans sa poitrine, ça se serre. L'envie et l'inquiétude se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont chaudes, Nino ? Un peu, maman. L'éclat de marelle tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les pierres de la cour sont froides. Un linge rouge bouge au vent. Un seau en métal sonne. Ça sent le café, près de la porte. Papa ouvre la porte de la cuisine. Tu as entendu le seau, Nino ? Oui, papa. Ça sonne. Le vent le touche. Un banc de bois attend au soleil. En ce moment, Nino joue. Chouchou joue avec lui. Ils sont dans la cour. Chouchou fait un gros câlin. Le câlin est trop fort. Nino est inquiet. C'est trop près. Sa poitrine est coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Nino recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le banc. Papa est l'adulte sur le banc. Papa, c'était trop. Je t'ai entendu. Tu as dit stop. Bravo, Nino. Tu as fait un pas vers le banc. Tu veux ta main dans ma main ? Oui, papa. Nino pose sa main dans la main de papa. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Chouchou pousse le seau tout doucement. Le seau sonne plus loin. La cour redevient calme. Le linge rouge claque une fois. Puis il se calme. Tu as vu le linge ? Oui. Il est rouge. Les pierres se réchauffent. Nino pose un pied dessus. Ce n'est plus froid. On reste sur le banc un moment ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un trait rose s'étire sur le sol chaud. Il est long, papa. Tu le vois, le trait ? Oui, papa. La poussière de craie pique le nez. J'ai tracé la marelle. Elle est grande, maman. Maman pose le caillou plat. Le caillou est chaud, un peu lisse. Il est chaud. Tu le touches, Nino ? Oui, du doigt. Sur une case, un &lt;emphasis level="moderate"&gt;éclat de marelle&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur la case ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur la craie. La craie gratte un peu. Elle gratte, papa. Tu t'accroupis, Nino ? Un peu. Une miette de craie dort au bord. Une miette, maman. Elle est sèche ? Oui. Le vent soulève un peu de poussière. Ça chatouille, papa. Tu l'entends, le vent ? Oui, il souffle. Une feuille tourne près des cases. Elle tourne. C'est le vent. Les pieds de Nino tapent le sol. Mes pieds, papa. Tu es bien prêt, Nino ? Oui, papa. Le sol de la marelle est rêche. Il est rêche. Aniss arrive près des cases. Ses baskets tapent la poussière. La marelle. Tu viens, Aniss ? Oui. Maman tend le caillou. Il tient chaud dans la paume. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. En ce moment, Nino lève le caillou. Tu le lances, Nino ? Oui, maman. Le caillou tape la première case. Moi aussi ! Aniss ouvre les bras tout grand. Il serre Nino très fort. Oh. Le sourire de Nino disparaît. Dans sa poitrine, ça se serre. L'envie et l'inquiétude se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont chaudes, Nino ? Un peu, maman. L'éclat de marelle tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Florian joue dans la cour. Un camarade le serre trop fort. Florian sent sa poitrine coincée. Il dit : je n'aime pas. C'est trop. Florian dit : &lt;emphasis&gt;stop&lt;/emphasis&gt;. Il recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le banc. Papa est l'adulte sur le banc. Florian va vers papa. Il dit : c'était trop. Papa l'écoute. Florian pose sa main dans la main de papa. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte.&lt;/slow&gt; [pause]</t>
+          <t>Un trait rose s'étire sur le sol chaud. Il est long, papa. Tu le vois, le trait ? Oui, papa. La poussière de craie pique le nez. J'ai tracé la marelle. Elle est grande, maman. Maman pose le caillou plat. Le caillou est chaud, un peu lisse. Il est chaud. Tu le touches, Nino ? Oui, du doigt. Sur une case, un &lt;emphasis&gt;éclat de marelle&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur la case ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur la craie. La craie gratte un peu. Elle gratte, papa. Tu t'accroupis, Nino ? Un peu. Une miette de craie dort au bord. Une miette, maman. Elle est sèche ? Oui. Le vent soulève un peu de poussière. Ça chatouille, papa. Tu l'entends, le vent ? Oui, il souffle. Une feuille tourne près des cases. Elle tourne. C'est le vent. Les pieds de Nino tapent le sol. Mes pieds, papa. Tu es bien prêt, Nino ? Oui, papa. Le sol de la marelle est rêche. Il est rêche. Aniss arrive près des cases. Ses baskets tapent la poussière. La marelle. Tu viens, Aniss ? Oui. Maman tend le caillou. Il tient chaud dans la paume. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. En ce moment, Nino lève le caillou. Tu le lances, Nino ? Oui, maman. Le caillou tape la première case. Moi aussi ! Aniss ouvre les bras tout grand. Il serre Nino très fort. Oh. Le sourire de Nino disparaît. Dans sa poitrine, ça se serre. L'envie et l'inquiétude se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont chaudes, Nino ? Un peu, maman. L'éclat de marelle tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>éclat de marelle</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,61 +1324,82 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_jouer_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les pierres de la cour sont froides.
-narrateur|Un linge rouge bouge au vent.
-narrateur|Un seau en métal sonne.
-narrateur|Ça sent le café, près de la porte.
-narrateur|Papa ouvre la porte de la cuisine.
-papa|Tu as entendu le seau, Nino ?
-enfant-m|Oui, papa. Ça sonne.
-papa|Le vent le touche.
-narrateur|Un banc de bois attend au soleil.
-narrateur|En ce moment, Nino joue.
-narrateur|Chouchou joue avec lui.
-narrateur|Ils sont dans la cour.
-narrateur|Chouchou fait un gros câlin.
-narrateur|Le câlin est trop fort.
-narrateur|Nino est inquiet.
-narrateur|C'est trop près.
-narrateur|Sa poitrine est coincée.
-narrateur|Ses épaules montent.
-enfant-m|Je n'aime pas.
-enfant-m|C'est trop.
-enfant-m|Stop.
-narrateur|Nino recule d'un pas.
-narrateur|Il peut s'éloigner.
-narrateur|Il s'éloigne vers le banc.
-narrateur|Papa est l'adulte sur le banc.
-enfant-m|Papa, c'était trop.
-papa|Je t'ai entendu.
-papa|Tu as dit stop.
-papa|Bravo, Nino.
-papa|Tu as fait un pas vers le banc.
-papa|Tu veux ta main dans ma main ?
+          <t>narrateur|Un trait rose s'étire sur le sol chaud.
+enfant-m|Il est long, papa.
+papa|Tu le vois, le trait ?
 enfant-m|Oui, papa.
-narrateur|Nino pose sa main dans la main de papa.
-narrateur|Il souffle.
-narrateur|Ses épaules descendent.
-papa|Dire stop, c'est permis.
-papa|On s'éloigne.
-papa|On va vers un adulte.
-narrateur|Chouchou pousse le seau tout doucement.
-narrateur|Le seau sonne plus loin.
-narrateur|La cour redevient calme.
-narrateur|Le linge rouge claque une fois.
-narrateur|Puis il se calme.
-papa|Tu as vu le linge ?
-enfant-m|Oui. Il est rouge.
-narrateur|Les pierres se réchauffent.
-narrateur|Nino pose un pied dessus.
-narrateur|Ce n'est plus froid.
-papa|On reste sur le banc un moment ?
-enfant-m|Oui, papa.</t>
+narrateur|La poussière de craie pique le nez.
+maman|J'ai tracé la marelle.
+enfant-m|Elle est grande, maman.
+narrateur|Maman pose le caillou plat.
+narrateur|Le caillou est chaud, un peu lisse.
+enfant-m|Il est chaud.
+papa|Tu le touches, Nino ?
+enfant-m|Oui, du doigt.
+narrateur|Sur une case, un éclat de marelle luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur la case ?
+enfant-m|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Un rayon glisse sur la craie.
+narrateur|La craie gratte un peu.
+enfant-m|Elle gratte, papa.
+maman|Tu t'accroupis, Nino ?
+enfant-m|Un peu.
+narrateur|Une miette de craie dort au bord.
+enfant-m|Une miette, maman.
+maman|Elle est sèche ?
+enfant-m|Oui.
+narrateur|Le vent soulève un peu de poussière.
+enfant-m|Ça chatouille, papa.
+papa|Tu l'entends, le vent ?
+enfant-m|Oui, il souffle.
+narrateur|Une feuille tourne près des cases.
+enfant-m|Elle tourne.
+maman|C'est le vent.
+narrateur|Les pieds de Nino tapent le sol.
+enfant-m|Mes pieds, papa.
+papa|Tu es bien prêt, Nino ?
+enfant-m|Oui, papa.
+narrateur|Le sol de la marelle est rêche.
+enfant-m|Il est rêche.
+narrateur|Aniss arrive près des cases.
+narrateur|Ses baskets tapent la poussière.
+copain|La marelle.
+enfant-m|Tu viens, Aniss ?
+copain|Oui.
+narrateur|Maman tend le caillou.
+narrateur|Il tient chaud dans la paume.
+enfant-m|Je veux jouer, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|En ce moment, Nino lève le caillou.
+maman|Tu le lances, Nino ?
+enfant-m|Oui, maman.
+narrateur|Le caillou tape la première case.
+copain|Moi aussi !
+narrateur|Aniss ouvre les bras tout grand.
+narrateur|Il serre Nino très fort.
+enfant-m|Oh.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, ça se serre.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|Ses épaules montent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Aniss, Nino ?
+enfant-m|Oui, papa.
+maman|Tes mains sont chaudes, Nino ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de marelle tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1415,12 +1436,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Nino. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est &lt;emphasis level="moderate"&gt;trop&lt;/emphasis&gt; pour Nino. Que dit-il ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est trop pour Florian. Que dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;C'est &lt;emphasis&gt;trop&lt;/emphasis&gt; pour Nino. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1483,7 +1504,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1494,7 +1515,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1509,34 +1530,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>trop</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1551,7 +1576,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1561,12 +1586,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=c_est_trop_pour_nino_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|C'est trop pour Nino. Que dit-il ?</t>
+          <t>narrateur|C'est trop pour Nino.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1593,17 +1619,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino a dit stop. Il a pu s'éloigner. Il a rejoint papa, l'adulte. Tu as dit stop. Bravo. Tu restes près du banc ? Oui. Le linge rouge bouge encore. Le café sent encore.</t>
+          <t>Nino veut jouer, tout de suite. Je lance, maintenant ! Il avance trop près d'Aniss. Les bras d'Aniss se referment. Viens. Nino ne peut plus souffler. Oh. Le sourire ne revient pas. Nino recule d'abord les épaules. Stop. Il recule d'un pas. Personne ne parle. Il observe le caillou, un instant. Il écoute le vent sur la craie. Tu veux jouer, Nino ? Papa reste à la même hauteur. Un peu loin. Loin ? Oui. Merci, Nino. Papa a vu les deux, près des cases. Le caillou colle un peu, sous les doigts. Il est chaud. Aniss lâche les bras. Nino pose le caillou. Case. Case, oui. Tu la vois, la case ? Oui, papa. Tu sautes, Nino ? J'y vais. Ils sautent la première case. Ça fait un petit bruit. Hop. Hop. C'est loin, la case ? Aniss ouvre la bouche. Loin. Nino garde un pas d'air. Un pas. Un pas, oui. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste près de la marelle ? Oui. Tes pieds sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino a dit stop. Il a pu s'éloigner. Il a rejoint papa, l'adulte. Tu as dit stop. Bravo. Tu restes près du banc ? Oui. Le linge rouge bouge encore. Le café sent encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino veut jouer, tout de suite. Je lance, maintenant ! Il avance trop près d'Aniss. Les bras d'Aniss se referment. Viens. Nino ne peut plus souffler. Oh. Le sourire ne revient pas. Nino recule d'abord les épaules. &lt;emphasis level="moderate"&gt;Stop&lt;/emphasis&gt;. Il recule d'un pas. Personne ne parle. Il observe le caillou, un instant. Il écoute le vent sur la craie. Tu veux jouer, Nino ? Papa reste à la même hauteur. Un peu loin. Loin ? Oui. Merci, Nino. Papa a vu les deux, près des cases. Le caillou colle un peu, sous les doigts. Il est chaud. Aniss lâche les bras. Nino pose le caillou. Case. Case, oui. Tu la vois, la case ? Oui, papa. Tu sautes, Nino ? J'y vais. Ils sautent la première case. Ça fait un petit bruit. Hop. Hop. C'est loin, la case ? Aniss ouvre la bouche. Loin. Nino garde un pas d'air. Un pas. Un pas, oui. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste près de la marelle ? Oui. Tes pieds sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Florian a dit &lt;emphasis&gt;stop&lt;/emphasis&gt;. Il a pu s'éloigner. Il rejoint papa, l'adulte.&lt;/slow&gt; [pause]</t>
+          <t>Nino veut jouer, tout de suite. Je lance, maintenant ! Il avance trop près d'Aniss. Les bras d'Aniss se referment. Viens. Nino ne peut plus souffler. Oh. Le sourire ne revient pas. Nino recule d'abord les épaules. &lt;emphasis&gt;Stop&lt;/emphasis&gt;. Il recule d'un pas. Personne ne parle. Il observe le caillou, un instant. Il écoute le vent sur la craie. Tu veux jouer, Nino ? Papa reste à la même hauteur. Un peu loin. Loin ? Oui. Merci, Nino. Papa a vu les deux, près des cases. Le caillou colle un peu, sous les doigts. Il est chaud. Aniss lâche les bras. Nino pose le caillou. Case. Case, oui. Tu la vois, la case ? Oui, papa. Tu sautes, Nino ? J'y vais. Ils sautent la première case. Ça fait un petit bruit. Hop. Hop. C'est loin, la case ? Aniss ouvre la bouche. Loin. Nino garde un pas d'air. Un pas. Un pas, oui. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste près de la marelle ? Oui. Tes pieds sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1650,18 +1676,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1684,30 +1710,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>Stop</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1716,10 +1742,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1728,24 +1754,62 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=gêne puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_dit_stop_il_recule; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino a dit stop.
-narrateur|Il a pu s'éloigner.
-narrateur|Il a rejoint papa, l'adulte.
-papa|Tu as dit stop.
-papa|Bravo.
-papa|Tu restes près du banc ?
+          <t>narrateur|Nino veut jouer, tout de suite.
+enfant-m|Je lance, maintenant !
+narrateur|Il avance trop près d'Aniss.
+narrateur|Les bras d'Aniss se referment.
+copain|Viens.
+narrateur|Nino ne peut plus souffler.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nino recule d'abord les épaules.
+enfant-m|Stop.
+narrateur|Il recule d'un pas.
+narrateur|Personne ne parle.
+narrateur|Il observe le caillou, un instant.
+narrateur|Il écoute le vent sur la craie.
+papa|Tu veux jouer, Nino ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Un peu loin.
+copain|Loin ?
 enfant-m|Oui.
-narrateur|Le linge rouge bouge encore.
-narrateur|Le café sent encore.</t>
+papa|Merci, Nino.
+narrateur|Papa a vu les deux, près des cases.
+maman|Le caillou colle un peu, sous les doigts.
+enfant-m|Il est chaud.
+narrateur|Aniss lâche les bras.
+narrateur|Nino pose le caillou.
+copain|Case.
+enfant-m|Case, oui.
+papa|Tu la vois, la case ?
+enfant-m|Oui, papa.
+maman|Tu sautes, Nino ?
+copain|J'y vais.
+narrateur|Ils sautent la première case.
+narrateur|Ça fait un petit bruit.
+enfant-m|Hop.
+copain|Hop.
+papa|C'est loin, la case ?
+narrateur|Aniss ouvre la bouche.
+copain|Loin.
+narrateur|Nino garde un pas d'air.
+copain|Un pas.
+enfant-m|Un pas, oui.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près de la marelle ?
+enfant-m|Oui.
+maman|Tes pieds sont au chaud ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
     </row>
@@ -1772,17 +1836,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino reste près du banc. Papa lui parle tout bas. Ta poitrine était coincée. Tu as écouté. Tu es plus calme, maintenant ? Oui, papa. Les pierres se réchauffent au soleil. Nino souffle encore une fois. Le seau en métal ne sonne plus. Chouchou s'assoit près du linge. Toi, tu restes sur le banc. Avec moi.</t>
+          <t>Maman pose la craie rose. La craie est un peu ronde. La case, maintenant ! Aniss lève le caillou. Loin. Le caillou glisse sur une case. Il glisse, maintenant ! Aniss attrape les épaules de Nino. Il serre trop, pour aider. Oh. Nino avance les bras, trop vite. Puis il s'arrête net. Stop. Il recule d'un pas, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la case, un instant. Il écoute le vent sur la craie. Sur la case, un éclat de marelle luit. Là, sur la case. Tu sautes, Aniss ? Aniss ne serre plus. Il souffle, puis recule. Il glisse. On pose le caillou ? Oui, papa. Nino pousse le caillou. Aniss le pose, sans se presser. Il tient. Il tient. La craie est chaude, Aniss ? Un peu. Tu sautes, Nino ? Oui, maman. Ils sautent près de la marelle. La poussière chatouille les chevilles. C'est plus facile. Le vent est calme ? Oui, papa. Un rayon passe sur la case. Il allume la marelle. Aniss souffle sur la craie. La craie. La craie, oui. La craie laisse un trait. Un trait rose.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino reste près du banc. Papa lui parle tout bas. Ta poitrine était coincée. Tu as écouté. Tu es plus calme, maintenant ? Oui, papa. Les pierres se réchauffent au soleil. Nino souffle encore une fois. Le seau en métal ne sonne plus. Chouchou s'assoit près du linge. Toi, tu restes sur le banc. Avec moi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pose la craie rose. La craie est un peu ronde. La case, maintenant ! Aniss lève le caillou. Loin. Le caillou glisse sur une case. Il glisse, maintenant ! Aniss attrape les épaules de Nino. Il serre trop, pour aider. Oh. Nino avance les bras, trop vite. Puis il s'arrête net. Stop. Il recule d'un pas, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la case, un instant. Il écoute le vent sur la craie. Sur la case, un &lt;emphasis level="moderate"&gt;éclat de marelle&lt;/emphasis&gt; luit. Là, sur la case. Tu sautes, Aniss ? Aniss ne serre plus. Il souffle, puis recule. Il glisse. On pose le caillou ? Oui, papa. Nino pousse le caillou. Aniss le pose, sans se presser. Il tient. Il tient. La craie est chaude, Aniss ? Un peu. Tu sautes, Nino ? Oui, maman. Ils sautent près de la marelle. La poussière chatouille les chevilles. C'est plus facile. Le vent est calme ? Oui, papa. Un rayon passe sur la case. Il allume la marelle. Aniss souffle sur la craie. La craie. La craie, oui. La craie laisse un trait. Un trait rose.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Florian reste près du banc. Papa lui parle tout bas.&lt;/slow&gt; [pause]</t>
+          <t>Maman pose la craie rose. La craie est un peu ronde. La case, maintenant ! Aniss lève le caillou. Loin. Le caillou glisse sur une case. Il glisse, maintenant ! Aniss attrape les épaules de Nino. Il serre trop, pour aider. Oh. Nino avance les bras, trop vite. Puis il s'arrête net. Stop. Il recule d'un pas, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la case, un instant. Il écoute le vent sur la craie. Sur la case, un &lt;emphasis&gt;éclat de marelle&lt;/emphasis&gt; luit. Là, sur la case. Tu sautes, Aniss ? Aniss ne serre plus. Il souffle, puis recule. Il glisse. On pose le caillou ? Oui, papa. Nino pousse le caillou. Aniss le pose, sans se presser. Il tient. Il tient. La craie est chaude, Aniss ? Un peu. Tu sautes, Nino ? Oui, maman. Ils sautent près de la marelle. La poussière chatouille les chevilles. C'est plus facile. Le vent est calme ? Oui, papa. Un rayon passe sur la case. Il allume la marelle. Aniss souffle sur la craie. La craie. La craie, oui. La craie laisse un trait. Un trait rose. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1829,18 +1893,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1861,28 +1925,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de marelle</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1891,10 +1959,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1903,23 +1971,61 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_caillou_glisse_aniss_serre_pour_aider; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino reste près du banc.
-narrateur|Papa lui parle tout bas.
-papa|Ta poitrine était coincée.
-papa|Tu as écouté.
-papa|Tu es plus calme, maintenant ?
+          <t>narrateur|Maman pose la craie rose.
+narrateur|La craie est un peu ronde.
+enfant-m|La case, maintenant !
+narrateur|Aniss lève le caillou.
+copain|Loin.
+narrateur|Le caillou glisse sur une case.
+enfant-m|Il glisse, maintenant !
+narrateur|Aniss attrape les épaules de Nino.
+narrateur|Il serre trop, pour aider.
+enfant-m|Oh.
+narrateur|Nino avance les bras, trop vite.
+narrateur|Puis il s'arrête net.
+enfant-m|Stop.
+narrateur|Il recule d'un pas, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la case, un instant.
+narrateur|Il écoute le vent sur la craie.
+narrateur|Sur la case, un éclat de marelle luit.
+enfant-m|Là, sur la case.
+enfant-m|Tu sautes, Aniss ?
+narrateur|Aniss ne serre plus.
+narrateur|Il souffle, puis recule.
+copain|Il glisse.
+papa|On pose le caillou ?
 enfant-m|Oui, papa.
-narrateur|Les pierres se réchauffent au soleil.
-narrateur|Nino souffle encore une fois.
-narrateur|Le seau en métal ne sonne plus.
-narrateur|Chouchou s'assoit près du linge.
-papa|Toi, tu restes sur le banc.
-papa|Avec moi.</t>
+narrateur|Nino pousse le caillou.
+narrateur|Aniss le pose, sans se presser.
+enfant-m|Il tient.
+copain|Il tient.
+papa|La craie est chaude, Aniss ?
+copain|Un peu.
+maman|Tu sautes, Nino ?
+enfant-m|Oui, maman.
+narrateur|Ils sautent près de la marelle.
+narrateur|La poussière chatouille les chevilles.
+enfant-m|C'est plus facile.
+papa|Le vent est calme ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur la case.
+enfant-m|Il allume la marelle.
+narrateur|Aniss souffle sur la craie.
+copain|La craie.
+enfant-m|La craie, oui.
+narrateur|La craie laisse un trait.
+enfant-m|Un trait rose.</t>
         </is>
       </c>
     </row>
@@ -1946,17 +2052,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloigné. Je suis allé vers papa. Bravo.</t>
+          <t>Ils restent près de la marelle. Maman essuie un peu de poussière. Le caillou a sauté, papa. Tu l'as vu, toi ? Oui, près des cases. On est bien, ici. Nino tapote le caillou du doigt. Il a une trace de craie. Tu la vois, la trace ? Oui, maman. Le caillou est resté, Nino. Oui, avec Aniss. Le caillou est resté. Ça sent la craie, un peu tiède. Et le soleil, maman. Oui, dans l'air. Le caillou reste sur une case. Un éclat de marelle tient sur la case.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloigné. Je suis allé vers papa. Bravo.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la marelle. Maman essuie un peu de poussière. Le caillou a sauté, papa. Tu l'as vu, toi ? Oui, près des cases. On est bien, ici. Nino tapote le caillou du doigt. Il a une trace de craie. Tu la vois, la trace ? Oui, maman. Le caillou est resté, Nino. Oui, avec Aniss. Le caillou est resté. Ça sent la craie, un peu tiède. Et le soleil, maman. Oui, dans l'air. Le caillou reste sur une case. Un &lt;emphasis level="moderate"&gt;éclat de marelle&lt;/emphasis&gt; tient sur la case.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la marelle. Maman essuie un peu de poussière. Le caillou a sauté, papa. Tu l'as vu, toi ? Oui, près des cases. On est bien, ici. Nino tapote le caillou du doigt. Il a une trace de craie. Tu la vois, la trace ? Oui, maman. Le caillou est resté, Nino. Oui, avec Aniss. Le caillou est resté. Ça sent la craie, un peu tiède. Et le soleil, maman. Oui, dans l'air. Le caillou reste sur une case. Un &lt;emphasis&gt;éclat de marelle&lt;/emphasis&gt; tient sur la case.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2003,7 +2109,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2011,7 +2117,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2023,12 +2129,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2037,14 +2143,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de marelle</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2056,11 +2166,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2069,27 +2179,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_case; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit stop.
-enfant-m|Je me suis éloigné.
-enfant-m|Je suis allé vers papa.
-papa|Bravo.</t>
+          <t>narrateur|Ils restent près de la marelle.
+narrateur|Maman essuie un peu de poussière.
+enfant-m|Le caillou a sauté, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près des cases.
+maman|On est bien, ici.
+narrateur|Nino tapote le caillou du doigt.
+enfant-m|Il a une trace de craie.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le caillou est resté, Nino.
+enfant-m|Oui, avec Aniss.
+copain|Le caillou est resté.
+narrateur|Ça sent la craie, un peu tiède.
+enfant-m|Et le soleil, maman.
+maman|Oui, dans l'air.
+narrateur|Le caillou reste sur une case.
+narrateur|Un éclat de marelle tient sur la case.</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2167,6 +2295,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>